<commit_message>
Doc: Write 'read-me' instructions
</commit_message>
<xml_diff>
--- a/data/data_preparation/experimental_data.xlsx
+++ b/data/data_preparation/experimental_data.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucas\PROJETOS\04_MD_VISCOSITY_GREEN_KUBO\data\data_preparation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49727363-6B82-4707-90B9-32DE1A9ADC97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F168E5BD-0E84-4CD1-8B93-9CEBA6748A7C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="RESULT" sheetId="3" r:id="rId1"/>
-    <sheet name="H2O" sheetId="1" r:id="rId2"/>
+    <sheet name="README" sheetId="4" r:id="rId1"/>
+    <sheet name="RESULT" sheetId="3" r:id="rId2"/>
+    <sheet name="H2O" sheetId="1" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="DadosExternos_1" localSheetId="0" hidden="1">RESULT!$A$1:$I$48</definedName>
+    <definedName name="DadosExternos_1" localSheetId="1" hidden="1">RESULT!$A$1:$I$48</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
   <extLst>
@@ -211,39 +212,6 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="25">
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -455,6 +423,39 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -471,6 +472,132 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>30480</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>45720</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="CaixaDeTexto 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1B62D8DB-5E20-4956-BA71-3149271DCB11}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="640080" y="327660"/>
+          <a:ext cx="4892040" cy="2232660"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:schemeClr val="lt1"/>
+        </a:solidFill>
+        <a:ln w="9525" cmpd="sng">
+          <a:solidFill>
+            <a:schemeClr val="lt1">
+              <a:shade val="50000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:lnRef>
+        <a:fillRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:scrgbClr r="0" g="0" b="0"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="dk1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:r>
+            <a:rPr lang="pt-BR" sz="1400" b="1"/>
+            <a:t>How to Use This Spreadsheet</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="pt-BR" b="1"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="pt-BR"/>
+            <a:t>The purpose of this spreadsheet is to normalize data provided in different units into the standard units required as input by the system.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="pt-BR"/>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="pt-BR"/>
+            <a:t>Update everything to process all tables and normalize them in the </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" b="1"/>
+            <a:t>RESULT</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR"/>
+            <a:t> tab.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:r>
+            <a:rPr lang="pt-BR"/>
+            <a:t>After making the changes, go to </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" b="1"/>
+            <a:t>Data → Refresh All</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR"/>
+            <a:t> in Excel to refresh all Power Query queries and connections at once. Then wait for the refresh process to finish completely before reviewing the </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR" b="1"/>
+            <a:t>RESULT</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="pt-BR"/>
+            <a:t> tab, as some queries may take a few moments to process.</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:endParaRPr lang="pt-BR" sz="1100"/>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -495,36 +622,36 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{79B1DAAA-0DC9-420F-ADA9-D9D9254762B4}" name="Systems_View" displayName="Systems_View" ref="A1:I48" tableType="queryTable" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
   <autoFilter ref="A1:I48" xr:uid="{79B1DAAA-0DC9-420F-ADA9-D9D9254762B4}"/>
   <tableColumns count="9">
-    <tableColumn id="10" xr3:uid="{287ED894-824A-4D02-8FEA-23DAA50B6B66}" uniqueName="10" name="SOLVENT" queryTableFieldId="1" dataDxfId="8"/>
-    <tableColumn id="2" xr3:uid="{D89CC5D5-30A2-4D4E-B21D-1085C4EEF539}" uniqueName="2" name="SOLUTE" queryTableFieldId="2" dataDxfId="7"/>
-    <tableColumn id="3" xr3:uid="{88A260A6-5FEE-4063-9B08-D74973B6A549}" uniqueName="3" name="PRESSURE_ATM" queryTableFieldId="3" dataDxfId="6"/>
-    <tableColumn id="4" xr3:uid="{0962C08C-347C-4AB7-A097-9404780D96FB}" uniqueName="4" name="TEMPERATURE_KELVIN" queryTableFieldId="4" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{47F7FF58-E3E1-4B14-92EE-E91499A61C44}" uniqueName="5" name="COMPOSITION_MOL_KG" queryTableFieldId="5" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{A72B8246-0C45-44EE-9204-98FB6CF9ADDB}" uniqueName="6" name="VISCOSITY_CP" queryTableFieldId="6" dataDxfId="3"/>
-    <tableColumn id="7" xr3:uid="{5E5EC9A9-2BB8-4676-BDCB-7C41C2EC62AC}" uniqueName="7" name="REFERENCE" queryTableFieldId="7" dataDxfId="2"/>
-    <tableColumn id="8" xr3:uid="{367C1B56-29C6-4294-9C46-3C0C50AF7265}" uniqueName="8" name="NOTE" queryTableFieldId="8" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{D452172E-C45D-4892-9966-989CD19A397F}" uniqueName="9" name="CREATED" queryTableFieldId="9" dataDxfId="0"/>
+    <tableColumn id="10" xr3:uid="{287ED894-824A-4D02-8FEA-23DAA50B6B66}" uniqueName="10" name="SOLVENT" queryTableFieldId="1" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{D89CC5D5-30A2-4D4E-B21D-1085C4EEF539}" uniqueName="2" name="SOLUTE" queryTableFieldId="2" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{88A260A6-5FEE-4063-9B08-D74973B6A549}" uniqueName="3" name="PRESSURE_ATM" queryTableFieldId="3" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{0962C08C-347C-4AB7-A097-9404780D96FB}" uniqueName="4" name="TEMPERATURE_KELVIN" queryTableFieldId="4" dataDxfId="19"/>
+    <tableColumn id="5" xr3:uid="{47F7FF58-E3E1-4B14-92EE-E91499A61C44}" uniqueName="5" name="COMPOSITION_MOL_KG" queryTableFieldId="5" dataDxfId="18"/>
+    <tableColumn id="6" xr3:uid="{A72B8246-0C45-44EE-9204-98FB6CF9ADDB}" uniqueName="6" name="VISCOSITY_CP" queryTableFieldId="6" dataDxfId="17"/>
+    <tableColumn id="7" xr3:uid="{5E5EC9A9-2BB8-4676-BDCB-7C41C2EC62AC}" uniqueName="7" name="REFERENCE" queryTableFieldId="7" dataDxfId="16"/>
+    <tableColumn id="8" xr3:uid="{367C1B56-29C6-4294-9C46-3C0C50AF7265}" uniqueName="8" name="NOTE" queryTableFieldId="8" dataDxfId="15"/>
+    <tableColumn id="9" xr3:uid="{D452172E-C45D-4892-9966-989CD19A397F}" uniqueName="9" name="CREATED" queryTableFieldId="9" dataDxfId="14"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F49ACE0F-ED39-479A-9BFD-04E71E3F30FB}" name="H2O" displayName="H2O" ref="A1:L48" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{F49ACE0F-ED39-479A-9BFD-04E71E3F30FB}" name="H2O" displayName="H2O" ref="A1:L48" totalsRowShown="0" headerRowDxfId="13" dataDxfId="12">
   <autoFilter ref="A1:L48" xr:uid="{F49ACE0F-ED39-479A-9BFD-04E71E3F30FB}"/>
   <tableColumns count="12">
-    <tableColumn id="1" xr3:uid="{CA9F4974-69F4-4772-90AC-88DDD1E08ABB}" name="SOLVENT" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{5F0B78F7-D5CF-4BBA-A5DE-2AAE4C4AA86A}" name="SOLUTE" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{7F729C42-0C81-4ACD-8069-536B007A51A7}" name="PRESSURE_VALUE" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{78C0A9F6-EC06-4C31-B0F0-4F7DC5D33896}" name="PRESSURE_UNIT" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{842D5E08-6B0D-482A-BDF3-FAF4C2ABF059}" name="TEMPERATURE_VALUE" dataDxfId="16"/>
-    <tableColumn id="6" xr3:uid="{884DB966-84EC-4FD5-AC80-9DDB8ECC6492}" name="TEMPERATURE_UNIT" dataDxfId="15"/>
-    <tableColumn id="7" xr3:uid="{681AAB4B-D571-43E1-8504-52E679EF1B51}" name="COMPOSITION_VALUE" dataDxfId="14"/>
-    <tableColumn id="8" xr3:uid="{C798AB0A-008F-4E9E-8AE8-5A4AD9FB3B71}" name="COMPOSITION_UNIT" dataDxfId="13"/>
-    <tableColumn id="9" xr3:uid="{E3406245-CBE4-40F6-9BAE-6361F6FB3BEB}" name="VISCOSITY_VALUE" dataDxfId="12"/>
-    <tableColumn id="10" xr3:uid="{F8006A84-F1BA-4FC2-8525-FAB29F7D1168}" name="VISCOSITY_UNIT" dataDxfId="11"/>
-    <tableColumn id="11" xr3:uid="{A2159BB3-BBE7-42B5-8C4E-8483E948CA45}" name="REFERENCE" dataDxfId="10"/>
-    <tableColumn id="12" xr3:uid="{1B6AE495-074C-4B19-A3E2-A6E25D7717EF}" name="NOTE" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{CA9F4974-69F4-4772-90AC-88DDD1E08ABB}" name="SOLVENT" dataDxfId="11"/>
+    <tableColumn id="2" xr3:uid="{5F0B78F7-D5CF-4BBA-A5DE-2AAE4C4AA86A}" name="SOLUTE" dataDxfId="10"/>
+    <tableColumn id="3" xr3:uid="{7F729C42-0C81-4ACD-8069-536B007A51A7}" name="PRESSURE_VALUE" dataDxfId="9"/>
+    <tableColumn id="4" xr3:uid="{78C0A9F6-EC06-4C31-B0F0-4F7DC5D33896}" name="PRESSURE_UNIT" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{842D5E08-6B0D-482A-BDF3-FAF4C2ABF059}" name="TEMPERATURE_VALUE" dataDxfId="7"/>
+    <tableColumn id="6" xr3:uid="{884DB966-84EC-4FD5-AC80-9DDB8ECC6492}" name="TEMPERATURE_UNIT" dataDxfId="6"/>
+    <tableColumn id="7" xr3:uid="{681AAB4B-D571-43E1-8504-52E679EF1B51}" name="COMPOSITION_VALUE" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{C798AB0A-008F-4E9E-8AE8-5A4AD9FB3B71}" name="COMPOSITION_UNIT" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{E3406245-CBE4-40F6-9BAE-6361F6FB3BEB}" name="VISCOSITY_VALUE" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{F8006A84-F1BA-4FC2-8525-FAB29F7D1168}" name="VISCOSITY_UNIT" dataDxfId="2"/>
+    <tableColumn id="11" xr3:uid="{A2159BB3-BBE7-42B5-8C4E-8483E948CA45}" name="REFERENCE" dataDxfId="1"/>
+    <tableColumn id="12" xr3:uid="{1B6AE495-074C-4B19-A3E2-A6E25D7717EF}" name="NOTE" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="0" showColumnStripes="0"/>
 </table>
@@ -792,6 +919,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1AE2C892-196A-4CBC-A84E-B26AB34C2169}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="2" customWidth="1"/>
+  </cols>
+  <sheetData/>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3BF6FD5-2701-4F97-B892-FE37BE990E49}">
   <dimension ref="A1:I48"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
@@ -2210,7 +2350,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:L48"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>

</xml_diff>